<commit_message>
Add uncategorized inventory export tooling and updated triage spreadsheets.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/sin-categoria-triage.xlsx
+++ b/exports/sin-categoria-triage.xlsx
@@ -1,13 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_838C7F541136A18BF615BA9C2D674DFEC6590D88" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Lists" state="veryHidden" r:id="rId4"/>
-    <sheet sheetId="2" name="Clover sin categoría (395)" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Productos a revisar (193)" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="LEER PRIMERO" state="visible" r:id="rId7"/>
+    <sheet name="Lists" sheetId="1" state="veryHidden" r:id="rId1"/>
+    <sheet name="Clover sin categoría (395)" sheetId="2" r:id="rId2"/>
+    <sheet name="Productos a revisar (193)" sheetId="3" r:id="rId3"/>
+    <sheet name="LEER PRIMERO" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -4345,17 +4349,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4719,9 +4725,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -4756,7 +4762,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -4764,7 +4770,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -4772,7 +4778,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -4780,7 +4786,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -4788,7 +4794,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -4796,7 +4802,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4804,46 +4810,46 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L396"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -19902,35 +19908,39 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="I10:I396">
-      <formula1>Lists!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="I2:I396">
-      <formula1>Lists!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="J10:J396">
-      <formula1>Lists!$B$1:$B$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="J2:J396">
-      <formula1>Lists!$B$1:$B$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="K10:K396">
-      <formula1>Lists!$C$1:$C$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="K2:K396">
-      <formula1>Lists!$C$1:$C$3</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0100-000000000000}">
+          <x14:formula1>
+            <xm:f>Lists!$A$1:$A$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I396</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0100-000002000000}">
+          <x14:formula1>
+            <xm:f>Lists!$B$1:$B$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>J2:J396</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0100-000004000000}">
+          <x14:formula1>
+            <xm:f>Lists!$C$1:$C$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>K2:K396</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L194"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -27313,35 +27323,39 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="I10:I194">
-      <formula1>Lists!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="I2:I194">
-      <formula1>Lists!$A$1:$A$15</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="J10:J194">
-      <formula1>Lists!$B$1:$B$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="J2:J194">
-      <formula1>Lists!$B$1:$B$9</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="K10:K194">
-      <formula1>Lists!$C$1:$C$3</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." sqref="K2:K194">
-      <formula1>Lists!$C$1:$C$3</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0200-000000000000}">
+          <x14:formula1>
+            <xm:f>Lists!$A$1:$A$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I194</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0200-000002000000}">
+          <x14:formula1>
+            <xm:f>Lists!$B$1:$B$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>J2:J194</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor inválido" error="Elige una opción de la lista." xr:uid="{00000000-0002-0000-0200-000004000000}">
+          <x14:formula1>
+            <xm:f>Lists!$C$1:$C$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>K2:K194</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -27371,7 +27385,7 @@
         <v>1437</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1438</v>
       </c>
@@ -27402,6 +27416,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>